<commit_message>
feat: agrega captura del reporte semaforizado y actualiza mocks
Output generado con datos ficticios procesados por AUDIBOT real.
Mocks v2 corregidos para ser compatibles con el parser de la app.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/input_cloudbeds_mock.xlsx
+++ b/samples/input_cloudbeds_mock.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002F4F4F"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,107 +416,107 @@
   <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Usuario</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Fecha y hora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fecha del servicio</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Habitación</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Apellido</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Núm. de reserva</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Código de la transacción</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Check-in</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Check-out</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Cant.</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Crédito</t>
         </is>
@@ -535,12 +525,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/03/2026 23:45</t>
+          <t>06/03/2026 23:10</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -560,27 +550,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rodríguez</t>
+          <t>Rodriguez</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>RES-10041</t>
+          <t>1001001001001</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CC_VISA</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Pago con Tarjeta Visa</t>
+          <t>VISA_CREDITO - Pago Registrada</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -590,15 +580,19 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Checked out</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+          <t>Checked Out</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>$85.000/TC 1420/VISA CREDITO 4134/CUPON 8801/LOTE 100</t>
+        </is>
+      </c>
       <c r="O2" t="n">
         <v>1</v>
       </c>
@@ -606,18 +600,18 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>85000</v>
+        <v>59.86</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/03/2026 23:46</t>
+          <t>06/03/2026 23:15</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -632,32 +626,32 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>María</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>López</t>
+          <t>Lopez</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>RES-10042</t>
+          <t>2002002002002</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>TRANSFER</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Transferencia Bancaria</t>
+          <t>TRANSFERENCIA - Pago Registrada</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -672,10 +666,14 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Checked out</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
+          <t>Checked Out</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>$120.000 TC 1420 TRANSFERENCIA</t>
+        </is>
+      </c>
       <c r="O3" t="n">
         <v>1</v>
       </c>
@@ -683,18 +681,18 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>120000</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/03/2026 23:47</t>
+          <t>06/03/2026 23:20</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -719,22 +717,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>RES-10043</t>
+          <t>3003003003003</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>USD_CASH</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Pago en efectivo USD</t>
+          <t>GREEN_CARD - Pago Registrada</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -749,10 +747,14 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Checked out</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
+          <t>Checked Out</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>$110.250 TC 1470 E4HOTELS</t>
+        </is>
+      </c>
       <c r="O4" t="n">
         <v>1</v>
       </c>
@@ -766,12 +768,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/03/2026 23:48</t>
+          <t>06/03/2026 23:25</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -791,27 +793,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Martínez</t>
+          <t>Martinez</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>RES-10044</t>
+          <t>4004004004004</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CC_MASTER</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Pago con Mastercard</t>
+          <t>MASTERCARD - Pago Registrada</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -826,10 +828,14 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Checked in</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
+          <t>In-House</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>$45.000/TC 1420/MASTER 5678/CUPON 8802/LOTE 100</t>
+        </is>
+      </c>
       <c r="O5" t="n">
         <v>1</v>
       </c>
@@ -837,18 +843,18 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>45000</v>
+        <v>31.69</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06/03/2026 23:49</t>
+          <t>06/03/2026 23:26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -868,27 +874,27 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Martínez</t>
+          <t>Martinez</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>RES-10044</t>
+          <t>4004004004004</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>CC_MASTER</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Pago con Mastercard (2do pago)</t>
+          <t>MASTERCARD - Pago Registrada</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -903,10 +909,14 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Checked in</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr"/>
+          <t>In-House</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>$55.000/TC 1420/MASTER 5678/CUPON 8803/LOTE 100</t>
+        </is>
+      </c>
       <c r="O6" t="n">
         <v>1</v>
       </c>
@@ -914,18 +924,18 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>55000</v>
+        <v>38.73</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06/03/2026 23:50</t>
+          <t>06/03/2026 23:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -945,27 +955,27 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Gómez</t>
+          <t>Gomez</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>RES-10045</t>
+          <t>5005005005005</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CC_VISA</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pago Visa — ANULADO</t>
+          <t>VISA_CREDITO - Pago Registrada</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -980,12 +990,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Checked out</t>
+          <t>Checked Out</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Anulación</t>
+          <t>$60.000/TC 1420/VISA 9012/CUPON 8804/LOTE 100</t>
         </is>
       </c>
       <c r="O7" t="n">
@@ -995,18 +1005,18 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>60000</v>
+        <v>42.25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/03/2026 23:50</t>
+          <t>06/03/2026 23:31</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1026,27 +1036,27 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Gómez</t>
+          <t>Gomez</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>RES-10045</t>
+          <t>5005005005005</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>REF-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>VOID</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Anulación Visa</t>
+          <t>VOID - anulación de pago</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1061,19 +1071,15 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Checked out</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Anulación</t>
-        </is>
-      </c>
+          <t>Checked Out</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
         <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>60000</v>
+        <v>42.25</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
@@ -1082,12 +1088,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>auditor01</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/03/2026 23:51</t>
+          <t>06/03/2026 23:40</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1107,27 +1113,27 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Fernández</t>
+          <t>Fernandez</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>RES-10046</t>
+          <t>6006006006006</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>PAY-CB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>TRANSFER</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Transferencia — Empresa XYZ</t>
+          <t>TRANSFERENCIA - Pago Registrada</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1142,10 +1148,14 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Checked out</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr"/>
+          <t>Checked Out</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>$98.500 TC 1420 TRANSFERENCIA EMPRESA XYZ</t>
+        </is>
+      </c>
       <c r="O9" t="n">
         <v>1</v>
       </c>
@@ -1153,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>98500</v>
+        <v>69.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>